<commit_message>
Change in company name
</commit_message>
<xml_diff>
--- a/Vendor_1.xlsx
+++ b/Vendor_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Agentic AI\Aerchain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950A55E2-7236-4139-AF75-8F4BAA80124F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC51158-0F81-4471-91A0-7D2E4AE05062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -270,7 +270,7 @@
     <t>Buyer reserves the right to split the award across multiple vendors</t>
   </si>
   <si>
-    <t>Max International</t>
+    <t>Max International - Vendor response</t>
   </si>
 </sst>
 </file>

</xml_diff>